<commit_message>
- added touched feature - made randomize feature consistant when turned on / off
</commit_message>
<xml_diff>
--- a/hmwebsite/modecraft/resources/data.xlsx
+++ b/hmwebsite/modecraft/resources/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\hmon.ir\hmwebsite\modecraft\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82B2126B-F1C1-4361-8BE3-C64E5E3120FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18FD58CA-3912-4F41-B5BF-0842E6C46646}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-315" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1260,7 +1260,9 @@
       <c r="D21" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="E21" s="8"/>
+      <c r="E21" s="8">
+        <v>110</v>
+      </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">

</xml_diff>